<commit_message>
Update test cases Excel file with new data
</commit_message>
<xml_diff>
--- a/Assignment 1 - Test cases.xlsx
+++ b/Assignment 1 - Test cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\test_automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3408D64-9F83-48A0-B8BC-8E927CB2AD86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ACBA3A3-F65D-4555-BD06-3B7E8C49D77E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="722" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="284">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -727,12 +727,6 @@
     <t>Evidence or rationale for the input type covered</t>
   </si>
   <si>
-    <t>Rationale: The input is a afternoon greeting</t>
-  </si>
-  <si>
-    <t>Rationale: The input contains the greeting "ayubowan" and a welcoming phrase</t>
-  </si>
-  <si>
     <t>Rationale: The overall message is a command/instruction</t>
   </si>
   <si>
@@ -817,9 +811,6 @@
     <t>Rationale: Input includes the numbers with the numeric suffix '100 n 80 k'</t>
   </si>
   <si>
-    <t>Rationale: Input includes the currency notation 'USD30 k'</t>
-  </si>
-  <si>
     <t>Rationale: Input includes the currency notation 'Rs.300,000'</t>
   </si>
   <si>
@@ -863,6 +854,24 @@
   </si>
   <si>
     <t>Rationale: Input includes multiple online identifiers including a  URL 'https://github.com/project/booking', email 'dev.student2026@gmail.com', and website 'www.smartbooking-docs.lk'</t>
+  </si>
+  <si>
+    <t>Student IT No: IT23345478</t>
+  </si>
+  <si>
+    <t>Student Name: Dissanayake D.M.C.C</t>
+  </si>
+  <si>
+    <t>Rationale: The input is a afternoon/night greeting</t>
+  </si>
+  <si>
+    <t>Rationale: The input contains the greeting "wewa!"</t>
+  </si>
+  <si>
+    <t>Rationale: Six consecutive English words "so let's go inside quickly" are inserted inside the Singlish input</t>
+  </si>
+  <si>
+    <t>Rationale: Input includes the currency notation 'USD30'</t>
   </si>
 </sst>
 </file>
@@ -986,9 +995,11 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1270,7 +1281,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:H54"/>
   <sheetFormatPr defaultRowHeight="49.95" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.88671875" customWidth="1"/>
@@ -1278,7 +1289,7 @@
     <col min="4" max="4" width="28.44140625" style="8" customWidth="1"/>
     <col min="5" max="5" width="26.5546875" customWidth="1"/>
     <col min="6" max="6" width="11.44140625" customWidth="1"/>
-    <col min="7" max="7" width="25.6640625" style="10" customWidth="1"/>
+    <col min="7" max="7" width="25.6640625" customWidth="1"/>
     <col min="8" max="8" width="40.77734375" style="8" customWidth="1"/>
     <col min="9" max="9" width="16" customWidth="1"/>
     <col min="10" max="11" width="12.33203125" customWidth="1"/>
@@ -1291,10 +1302,10 @@
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
@@ -1332,7 +1343,7 @@
       <c r="G2" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="H2" s="11" t="s">
+      <c r="H2" s="10" t="s">
         <v>233</v>
       </c>
     </row>
@@ -1358,7 +1369,7 @@
       <c r="G3" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="H3" s="11" t="s">
+      <c r="H3" s="10" t="s">
         <v>233</v>
       </c>
     </row>
@@ -1384,7 +1395,7 @@
       <c r="G4" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="H4" s="11" t="s">
+      <c r="H4" s="10" t="s">
         <v>233</v>
       </c>
     </row>
@@ -1410,8 +1421,8 @@
       <c r="G5" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="H5" s="11" t="s">
-        <v>235</v>
+      <c r="H5" s="10" t="s">
+        <v>280</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1436,8 +1447,8 @@
       <c r="G6" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="H6" s="11" t="s">
-        <v>236</v>
+      <c r="H6" s="10" t="s">
+        <v>281</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1462,8 +1473,8 @@
       <c r="G7" s="9" t="s">
         <v>211</v>
       </c>
-      <c r="H7" s="11" t="s">
-        <v>237</v>
+      <c r="H7" s="10" t="s">
+        <v>235</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1488,8 +1499,8 @@
       <c r="G8" s="9" t="s">
         <v>211</v>
       </c>
-      <c r="H8" s="11" t="s">
-        <v>238</v>
+      <c r="H8" s="10" t="s">
+        <v>236</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1514,8 +1525,8 @@
       <c r="G9" s="9" t="s">
         <v>212</v>
       </c>
-      <c r="H9" s="11" t="s">
-        <v>241</v>
+      <c r="H9" s="10" t="s">
+        <v>239</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1540,8 +1551,8 @@
       <c r="G10" s="9" t="s">
         <v>212</v>
       </c>
-      <c r="H10" s="11" t="s">
-        <v>239</v>
+      <c r="H10" s="10" t="s">
+        <v>237</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1566,8 +1577,8 @@
       <c r="G11" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="H11" s="11" t="s">
-        <v>242</v>
+      <c r="H11" s="10" t="s">
+        <v>240</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1592,8 +1603,8 @@
       <c r="G12" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="H12" s="11" t="s">
-        <v>242</v>
+      <c r="H12" s="10" t="s">
+        <v>240</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1618,8 +1629,8 @@
       <c r="G13" s="9" t="s">
         <v>214</v>
       </c>
-      <c r="H13" s="11" t="s">
-        <v>240</v>
+      <c r="H13" s="10" t="s">
+        <v>238</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1644,8 +1655,8 @@
       <c r="G14" s="9" t="s">
         <v>214</v>
       </c>
-      <c r="H14" s="11" t="s">
-        <v>243</v>
+      <c r="H14" s="10" t="s">
+        <v>241</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1670,8 +1681,8 @@
       <c r="G15" s="9" t="s">
         <v>215</v>
       </c>
-      <c r="H15" s="11" t="s">
-        <v>244</v>
+      <c r="H15" s="10" t="s">
+        <v>242</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1696,8 +1707,8 @@
       <c r="G16" s="9" t="s">
         <v>215</v>
       </c>
-      <c r="H16" s="11" t="s">
-        <v>245</v>
+      <c r="H16" s="10" t="s">
+        <v>243</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1722,8 +1733,8 @@
       <c r="G17" s="9" t="s">
         <v>216</v>
       </c>
-      <c r="H17" s="11" t="s">
-        <v>246</v>
+      <c r="H17" s="10" t="s">
+        <v>244</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1748,8 +1759,8 @@
       <c r="G18" s="9" t="s">
         <v>216</v>
       </c>
-      <c r="H18" s="11" t="s">
-        <v>247</v>
+      <c r="H18" s="10" t="s">
+        <v>245</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1774,8 +1785,8 @@
       <c r="G19" s="9" t="s">
         <v>217</v>
       </c>
-      <c r="H19" s="11" t="s">
-        <v>248</v>
+      <c r="H19" s="10" t="s">
+        <v>246</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1800,8 +1811,8 @@
       <c r="G20" s="9" t="s">
         <v>217</v>
       </c>
-      <c r="H20" s="11" t="s">
-        <v>249</v>
+      <c r="H20" s="10" t="s">
+        <v>247</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1826,8 +1837,8 @@
       <c r="G21" s="9" t="s">
         <v>218</v>
       </c>
-      <c r="H21" s="11" t="s">
-        <v>250</v>
+      <c r="H21" s="10" t="s">
+        <v>248</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1852,8 +1863,8 @@
       <c r="G22" s="9" t="s">
         <v>218</v>
       </c>
-      <c r="H22" s="11" t="s">
-        <v>250</v>
+      <c r="H22" s="10" t="s">
+        <v>282</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1878,8 +1889,8 @@
       <c r="G23" s="9" t="s">
         <v>219</v>
       </c>
-      <c r="H23" s="11" t="s">
-        <v>252</v>
+      <c r="H23" s="10" t="s">
+        <v>250</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1904,8 +1915,8 @@
       <c r="G24" s="9" t="s">
         <v>219</v>
       </c>
-      <c r="H24" s="11" t="s">
-        <v>251</v>
+      <c r="H24" s="10" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1930,8 +1941,8 @@
       <c r="G25" s="9" t="s">
         <v>220</v>
       </c>
-      <c r="H25" s="11" t="s">
-        <v>254</v>
+      <c r="H25" s="10" t="s">
+        <v>252</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1956,8 +1967,8 @@
       <c r="G26" s="9" t="s">
         <v>220</v>
       </c>
-      <c r="H26" s="11" t="s">
-        <v>253</v>
+      <c r="H26" s="10" t="s">
+        <v>251</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1982,8 +1993,8 @@
       <c r="G27" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="H27" s="11" t="s">
-        <v>256</v>
+      <c r="H27" s="10" t="s">
+        <v>254</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -2008,8 +2019,8 @@
       <c r="G28" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="H28" s="11" t="s">
-        <v>255</v>
+      <c r="H28" s="10" t="s">
+        <v>253</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -2034,8 +2045,8 @@
       <c r="G29" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="H29" s="11" t="s">
-        <v>257</v>
+      <c r="H29" s="10" t="s">
+        <v>255</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -2060,8 +2071,8 @@
       <c r="G30" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="H30" s="11" t="s">
-        <v>258</v>
+      <c r="H30" s="10" t="s">
+        <v>256</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -2086,8 +2097,8 @@
       <c r="G31" s="9" t="s">
         <v>223</v>
       </c>
-      <c r="H31" s="11" t="s">
-        <v>259</v>
+      <c r="H31" s="10" t="s">
+        <v>257</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -2112,8 +2123,8 @@
       <c r="G32" s="9" t="s">
         <v>223</v>
       </c>
-      <c r="H32" s="11" t="s">
-        <v>260</v>
+      <c r="H32" s="10" t="s">
+        <v>258</v>
       </c>
     </row>
     <row r="33" spans="1:8" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -2138,8 +2149,8 @@
       <c r="G33" s="9" t="s">
         <v>224</v>
       </c>
-      <c r="H33" s="11" t="s">
-        <v>261</v>
+      <c r="H33" s="10" t="s">
+        <v>259</v>
       </c>
     </row>
     <row r="34" spans="1:8" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -2164,8 +2175,8 @@
       <c r="G34" s="9" t="s">
         <v>224</v>
       </c>
-      <c r="H34" s="11" t="s">
-        <v>262</v>
+      <c r="H34" s="10" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="35" spans="1:8" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -2190,8 +2201,8 @@
       <c r="G35" s="9" t="s">
         <v>225</v>
       </c>
-      <c r="H35" s="11" t="s">
-        <v>263</v>
+      <c r="H35" s="10" t="s">
+        <v>261</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -2216,8 +2227,8 @@
       <c r="G36" s="9" t="s">
         <v>225</v>
       </c>
-      <c r="H36" s="11" t="s">
-        <v>264</v>
+      <c r="H36" s="10" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -2242,8 +2253,8 @@
       <c r="G37" s="9" t="s">
         <v>226</v>
       </c>
-      <c r="H37" s="11" t="s">
-        <v>265</v>
+      <c r="H37" s="10" t="s">
+        <v>283</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -2268,8 +2279,8 @@
       <c r="G38" s="9" t="s">
         <v>226</v>
       </c>
-      <c r="H38" s="11" t="s">
-        <v>266</v>
+      <c r="H38" s="10" t="s">
+        <v>263</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -2294,8 +2305,8 @@
       <c r="G39" s="9" t="s">
         <v>227</v>
       </c>
-      <c r="H39" s="11" t="s">
-        <v>267</v>
+      <c r="H39" s="10" t="s">
+        <v>264</v>
       </c>
     </row>
     <row r="40" spans="1:8" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -2320,8 +2331,8 @@
       <c r="G40" s="9" t="s">
         <v>227</v>
       </c>
-      <c r="H40" s="11" t="s">
-        <v>268</v>
+      <c r="H40" s="10" t="s">
+        <v>265</v>
       </c>
     </row>
     <row r="41" spans="1:8" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -2346,8 +2357,8 @@
       <c r="G41" s="9" t="s">
         <v>228</v>
       </c>
-      <c r="H41" s="11" t="s">
-        <v>270</v>
+      <c r="H41" s="10" t="s">
+        <v>267</v>
       </c>
     </row>
     <row r="42" spans="1:8" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -2372,8 +2383,8 @@
       <c r="G42" s="9" t="s">
         <v>228</v>
       </c>
-      <c r="H42" s="11" t="s">
-        <v>269</v>
+      <c r="H42" s="10" t="s">
+        <v>266</v>
       </c>
     </row>
     <row r="43" spans="1:8" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -2384,7 +2395,7 @@
         <v>13</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="D43" s="6" t="s">
         <v>173</v>
@@ -2398,8 +2409,8 @@
       <c r="G43" s="9" t="s">
         <v>229</v>
       </c>
-      <c r="H43" s="11" t="s">
-        <v>271</v>
+      <c r="H43" s="10" t="s">
+        <v>268</v>
       </c>
     </row>
     <row r="44" spans="1:8" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -2424,8 +2435,8 @@
       <c r="G44" s="9" t="s">
         <v>229</v>
       </c>
-      <c r="H44" s="11" t="s">
-        <v>273</v>
+      <c r="H44" s="10" t="s">
+        <v>270</v>
       </c>
     </row>
     <row r="45" spans="1:8" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -2450,8 +2461,8 @@
       <c r="G45" s="9" t="s">
         <v>230</v>
       </c>
-      <c r="H45" s="11" t="s">
-        <v>274</v>
+      <c r="H45" s="10" t="s">
+        <v>271</v>
       </c>
     </row>
     <row r="46" spans="1:8" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -2476,8 +2487,8 @@
       <c r="G46" s="9" t="s">
         <v>230</v>
       </c>
-      <c r="H46" s="11" t="s">
-        <v>275</v>
+      <c r="H46" s="10" t="s">
+        <v>272</v>
       </c>
     </row>
     <row r="47" spans="1:8" ht="73.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -2502,8 +2513,8 @@
       <c r="G47" s="9" t="s">
         <v>231</v>
       </c>
-      <c r="H47" s="11" t="s">
-        <v>276</v>
+      <c r="H47" s="10" t="s">
+        <v>273</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="81.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
@@ -2528,8 +2539,8 @@
       <c r="G48" s="9" t="s">
         <v>231</v>
       </c>
-      <c r="H48" s="11" t="s">
-        <v>277</v>
+      <c r="H48" s="10" t="s">
+        <v>274</v>
       </c>
     </row>
     <row r="49" spans="1:8" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -2554,8 +2565,8 @@
       <c r="G49" s="9" t="s">
         <v>232</v>
       </c>
-      <c r="H49" s="11" t="s">
-        <v>278</v>
+      <c r="H49" s="10" t="s">
+        <v>275</v>
       </c>
     </row>
     <row r="50" spans="1:8" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -2580,8 +2591,8 @@
       <c r="G50" s="9" t="s">
         <v>232</v>
       </c>
-      <c r="H50" s="11" t="s">
-        <v>279</v>
+      <c r="H50" s="10" t="s">
+        <v>276</v>
       </c>
     </row>
     <row r="51" spans="1:8" ht="150" customHeight="1" x14ac:dyDescent="0.3">
@@ -2606,11 +2617,29 @@
       <c r="G51" s="9" t="s">
         <v>231</v>
       </c>
-      <c r="H51" s="11" t="s">
-        <v>280</v>
-      </c>
+      <c r="H51" s="10" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="11" t="s">
+        <v>278</v>
+      </c>
+      <c r="B53" s="11"/>
+      <c r="C53" s="11"/>
+    </row>
+    <row r="54" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="11" t="s">
+        <v>279</v>
+      </c>
+      <c r="B54" s="11"/>
+      <c r="C54" s="11"/>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A53:C53"/>
+    <mergeCell ref="A54:C54"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>